<commit_message>
23.07. commit 2 Vlada
</commit_message>
<xml_diff>
--- a/results/TestResults.xlsx
+++ b/results/TestResults.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="205">
   <si>
     <t>App</t>
   </si>
@@ -537,6 +537,111 @@
   </si>
   <si>
     <t>23.07.2026:07:25</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:07:47</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_23_07_2026_07_47.jpg</t>
+  </si>
+  <si>
+    <t>23.07.2026:07:55</t>
+  </si>
+  <si>
+    <t>23.07.2026:08:19</t>
+  </si>
+  <si>
+    <t>23.07.2026:08:23</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model11_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:08:32</t>
+  </si>
+  <si>
+    <t>23.07.2026:08:59</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model11_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:02</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:13</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:14</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_Invalid_Bez_Poziva_Na_Broj_[WEB]_23_07_2026_09_14.jpg</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:15</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model97_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:26</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Purpose_Code_289_Invalid_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:32</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:42</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]_23_07_2026_09_42.jpg</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:47</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]_23_07_2026_09_47.jpg</t>
+  </si>
+  <si>
+    <t>23.07.2026:09:49</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Model97_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:10:03</t>
+  </si>
+  <si>
+    <t>23.07.2026:10:05</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_Budzetski_Non_Urgent_Payment_Model97_[WEB]</t>
+  </si>
+  <si>
+    <t>23.07.2026:10:16</t>
+  </si>
+  <si>
+    <t>23.07.2026:10:18</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model97_[WEB]_23_07_2026_10_18.jpg</t>
+  </si>
+  <si>
+    <t>23.07.2026:10:20</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model11_[WEB]_23_07_2026_10_20.jpg</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1297,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="595">
+  <cellXfs count="775">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1794,6 +1899,186 @@
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2962,7 +3247,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XFD67"/>
+  <dimension ref="A1:XFD87"/>
   <sheetFormatPr defaultColWidth="8.82407407407407" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="9.33333333333333" collapsed="true"/>
@@ -21295,6 +21580,586 @@
         <v>14</v>
       </c>
     </row>
+    <row r="68">
+      <c r="B68" t="s" s="595">
+        <v>170</v>
+      </c>
+      <c r="C68" t="s" s="596">
+        <v>11</v>
+      </c>
+      <c r="D68" t="s" s="597">
+        <v>171</v>
+      </c>
+      <c r="E68" t="s" s="598">
+        <v>13</v>
+      </c>
+      <c r="F68" t="s" s="599">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s" s="600">
+        <v>149</v>
+      </c>
+      <c r="H68" t="s" s="601">
+        <v>14</v>
+      </c>
+      <c r="I68" t="s" s="602">
+        <v>17</v>
+      </c>
+      <c r="J68" t="s" s="603">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="s" s="604">
+        <v>170</v>
+      </c>
+      <c r="C69" t="s" s="605">
+        <v>38</v>
+      </c>
+      <c r="D69" t="s" s="606">
+        <v>173</v>
+      </c>
+      <c r="E69" t="s" s="607">
+        <v>13</v>
+      </c>
+      <c r="F69" t="s" s="608">
+        <v>14</v>
+      </c>
+      <c r="G69" t="s" s="609">
+        <v>149</v>
+      </c>
+      <c r="H69" t="s" s="610">
+        <v>14</v>
+      </c>
+      <c r="I69" t="s" s="611">
+        <v>17</v>
+      </c>
+      <c r="J69" t="s" s="612">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="s" s="613">
+        <v>170</v>
+      </c>
+      <c r="C70" t="s" s="614">
+        <v>38</v>
+      </c>
+      <c r="D70" t="s" s="615">
+        <v>174</v>
+      </c>
+      <c r="E70" t="s" s="616">
+        <v>13</v>
+      </c>
+      <c r="F70" t="s" s="617">
+        <v>14</v>
+      </c>
+      <c r="G70" t="s" s="618">
+        <v>149</v>
+      </c>
+      <c r="H70" t="s" s="619">
+        <v>14</v>
+      </c>
+      <c r="I70" t="s" s="620">
+        <v>17</v>
+      </c>
+      <c r="J70" t="s" s="621">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="s" s="622">
+        <v>166</v>
+      </c>
+      <c r="C71" t="s" s="623">
+        <v>38</v>
+      </c>
+      <c r="D71" t="s" s="624">
+        <v>175</v>
+      </c>
+      <c r="E71" t="s" s="625">
+        <v>13</v>
+      </c>
+      <c r="F71" t="s" s="626">
+        <v>14</v>
+      </c>
+      <c r="G71" t="s" s="627">
+        <v>149</v>
+      </c>
+      <c r="H71" t="s" s="628">
+        <v>14</v>
+      </c>
+      <c r="I71" t="s" s="629">
+        <v>17</v>
+      </c>
+      <c r="J71" t="s" s="630">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="s" s="631">
+        <v>176</v>
+      </c>
+      <c r="C72" t="s" s="632">
+        <v>38</v>
+      </c>
+      <c r="D72" t="s" s="633">
+        <v>177</v>
+      </c>
+      <c r="E72" t="s" s="634">
+        <v>13</v>
+      </c>
+      <c r="F72" t="s" s="635">
+        <v>14</v>
+      </c>
+      <c r="G72" t="s" s="636">
+        <v>149</v>
+      </c>
+      <c r="H72" t="s" s="637">
+        <v>14</v>
+      </c>
+      <c r="I72" t="s" s="638">
+        <v>17</v>
+      </c>
+      <c r="J72" t="s" s="639">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="s" s="640">
+        <v>176</v>
+      </c>
+      <c r="C73" t="s" s="641">
+        <v>38</v>
+      </c>
+      <c r="D73" t="s" s="642">
+        <v>178</v>
+      </c>
+      <c r="E73" t="s" s="643">
+        <v>13</v>
+      </c>
+      <c r="F73" t="s" s="644">
+        <v>14</v>
+      </c>
+      <c r="G73" t="s" s="645">
+        <v>149</v>
+      </c>
+      <c r="H73" t="s" s="646">
+        <v>14</v>
+      </c>
+      <c r="I73" t="s" s="647">
+        <v>17</v>
+      </c>
+      <c r="J73" t="s" s="648">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="s" s="649">
+        <v>179</v>
+      </c>
+      <c r="C74" t="s" s="650">
+        <v>38</v>
+      </c>
+      <c r="D74" t="s" s="651">
+        <v>180</v>
+      </c>
+      <c r="E74" t="s" s="652">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s" s="653">
+        <v>14</v>
+      </c>
+      <c r="G74" t="s" s="654">
+        <v>149</v>
+      </c>
+      <c r="H74" t="s" s="655">
+        <v>14</v>
+      </c>
+      <c r="I74" t="s" s="656">
+        <v>17</v>
+      </c>
+      <c r="J74" t="s" s="657">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="s" s="658">
+        <v>176</v>
+      </c>
+      <c r="C75" t="s" s="659">
+        <v>38</v>
+      </c>
+      <c r="D75" t="s" s="660">
+        <v>181</v>
+      </c>
+      <c r="E75" t="s" s="661">
+        <v>13</v>
+      </c>
+      <c r="F75" t="s" s="662">
+        <v>14</v>
+      </c>
+      <c r="G75" t="s" s="663">
+        <v>149</v>
+      </c>
+      <c r="H75" t="s" s="664">
+        <v>14</v>
+      </c>
+      <c r="I75" t="s" s="665">
+        <v>17</v>
+      </c>
+      <c r="J75" t="s" s="666">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="s" s="667">
+        <v>182</v>
+      </c>
+      <c r="C76" t="s" s="668">
+        <v>11</v>
+      </c>
+      <c r="D76" t="s" s="669">
+        <v>183</v>
+      </c>
+      <c r="E76" t="s" s="670">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s" s="671">
+        <v>14</v>
+      </c>
+      <c r="G76" t="s" s="672">
+        <v>149</v>
+      </c>
+      <c r="H76" t="s" s="673">
+        <v>14</v>
+      </c>
+      <c r="I76" t="s" s="674">
+        <v>17</v>
+      </c>
+      <c r="J76" t="s" s="675">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="s" s="676">
+        <v>182</v>
+      </c>
+      <c r="C77" t="s" s="677">
+        <v>38</v>
+      </c>
+      <c r="D77" t="s" s="678">
+        <v>185</v>
+      </c>
+      <c r="E77" t="s" s="679">
+        <v>13</v>
+      </c>
+      <c r="F77" t="s" s="680">
+        <v>14</v>
+      </c>
+      <c r="G77" t="s" s="681">
+        <v>149</v>
+      </c>
+      <c r="H77" t="s" s="682">
+        <v>14</v>
+      </c>
+      <c r="I77" t="s" s="683">
+        <v>17</v>
+      </c>
+      <c r="J77" t="s" s="684">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="s" s="685">
+        <v>186</v>
+      </c>
+      <c r="C78" t="s" s="686">
+        <v>38</v>
+      </c>
+      <c r="D78" t="s" s="687">
+        <v>187</v>
+      </c>
+      <c r="E78" t="s" s="688">
+        <v>13</v>
+      </c>
+      <c r="F78" t="s" s="689">
+        <v>14</v>
+      </c>
+      <c r="G78" t="s" s="690">
+        <v>149</v>
+      </c>
+      <c r="H78" t="s" s="691">
+        <v>14</v>
+      </c>
+      <c r="I78" t="s" s="692">
+        <v>17</v>
+      </c>
+      <c r="J78" t="s" s="693">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="s" s="694">
+        <v>188</v>
+      </c>
+      <c r="C79" t="s" s="695">
+        <v>38</v>
+      </c>
+      <c r="D79" t="s" s="696">
+        <v>189</v>
+      </c>
+      <c r="E79" t="s" s="697">
+        <v>13</v>
+      </c>
+      <c r="F79" t="s" s="698">
+        <v>14</v>
+      </c>
+      <c r="G79" t="s" s="699">
+        <v>149</v>
+      </c>
+      <c r="H79" t="s" s="700">
+        <v>14</v>
+      </c>
+      <c r="I79" t="s" s="701">
+        <v>17</v>
+      </c>
+      <c r="J79" t="s" s="702">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="s" s="703">
+        <v>190</v>
+      </c>
+      <c r="C80" t="s" s="704">
+        <v>11</v>
+      </c>
+      <c r="D80" t="s" s="705">
+        <v>191</v>
+      </c>
+      <c r="E80" t="s" s="706">
+        <v>13</v>
+      </c>
+      <c r="F80" t="s" s="707">
+        <v>14</v>
+      </c>
+      <c r="G80" t="s" s="708">
+        <v>149</v>
+      </c>
+      <c r="H80" t="s" s="709">
+        <v>14</v>
+      </c>
+      <c r="I80" t="s" s="710">
+        <v>17</v>
+      </c>
+      <c r="J80" t="s" s="711">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="s" s="712">
+        <v>190</v>
+      </c>
+      <c r="C81" t="s" s="713">
+        <v>11</v>
+      </c>
+      <c r="D81" t="s" s="714">
+        <v>193</v>
+      </c>
+      <c r="E81" t="s" s="715">
+        <v>13</v>
+      </c>
+      <c r="F81" t="s" s="716">
+        <v>14</v>
+      </c>
+      <c r="G81" t="s" s="717">
+        <v>149</v>
+      </c>
+      <c r="H81" t="s" s="718">
+        <v>14</v>
+      </c>
+      <c r="I81" t="s" s="719">
+        <v>17</v>
+      </c>
+      <c r="J81" t="s" s="720">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="s" s="721">
+        <v>190</v>
+      </c>
+      <c r="C82" t="s" s="722">
+        <v>38</v>
+      </c>
+      <c r="D82" t="s" s="723">
+        <v>195</v>
+      </c>
+      <c r="E82" t="s" s="724">
+        <v>13</v>
+      </c>
+      <c r="F82" t="s" s="725">
+        <v>14</v>
+      </c>
+      <c r="G82" t="s" s="726">
+        <v>149</v>
+      </c>
+      <c r="H82" t="s" s="727">
+        <v>14</v>
+      </c>
+      <c r="I82" t="s" s="728">
+        <v>17</v>
+      </c>
+      <c r="J82" t="s" s="729">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="s" s="730">
+        <v>196</v>
+      </c>
+      <c r="C83" t="s" s="731">
+        <v>38</v>
+      </c>
+      <c r="D83" t="s" s="732">
+        <v>197</v>
+      </c>
+      <c r="E83" t="s" s="733">
+        <v>13</v>
+      </c>
+      <c r="F83" t="s" s="734">
+        <v>14</v>
+      </c>
+      <c r="G83" t="s" s="735">
+        <v>149</v>
+      </c>
+      <c r="H83" t="s" s="736">
+        <v>14</v>
+      </c>
+      <c r="I83" t="s" s="737">
+        <v>17</v>
+      </c>
+      <c r="J83" t="s" s="738">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="s" s="739">
+        <v>196</v>
+      </c>
+      <c r="C84" t="s" s="740">
+        <v>38</v>
+      </c>
+      <c r="D84" t="s" s="741">
+        <v>198</v>
+      </c>
+      <c r="E84" t="s" s="742">
+        <v>13</v>
+      </c>
+      <c r="F84" t="s" s="743">
+        <v>14</v>
+      </c>
+      <c r="G84" t="s" s="744">
+        <v>149</v>
+      </c>
+      <c r="H84" t="s" s="745">
+        <v>14</v>
+      </c>
+      <c r="I84" t="s" s="746">
+        <v>17</v>
+      </c>
+      <c r="J84" t="s" s="747">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="s" s="748">
+        <v>199</v>
+      </c>
+      <c r="C85" t="s" s="749">
+        <v>38</v>
+      </c>
+      <c r="D85" t="s" s="750">
+        <v>200</v>
+      </c>
+      <c r="E85" t="s" s="751">
+        <v>13</v>
+      </c>
+      <c r="F85" t="s" s="752">
+        <v>14</v>
+      </c>
+      <c r="G85" t="s" s="753">
+        <v>149</v>
+      </c>
+      <c r="H85" t="s" s="754">
+        <v>14</v>
+      </c>
+      <c r="I85" t="s" s="755">
+        <v>17</v>
+      </c>
+      <c r="J85" t="s" s="756">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="s" s="757">
+        <v>186</v>
+      </c>
+      <c r="C86" t="s" s="758">
+        <v>11</v>
+      </c>
+      <c r="D86" t="s" s="759">
+        <v>201</v>
+      </c>
+      <c r="E86" t="s" s="760">
+        <v>13</v>
+      </c>
+      <c r="F86" t="s" s="761">
+        <v>14</v>
+      </c>
+      <c r="G86" t="s" s="762">
+        <v>149</v>
+      </c>
+      <c r="H86" t="s" s="763">
+        <v>14</v>
+      </c>
+      <c r="I86" t="s" s="764">
+        <v>17</v>
+      </c>
+      <c r="J86" t="s" s="765">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="s" s="766">
+        <v>179</v>
+      </c>
+      <c r="C87" t="s" s="767">
+        <v>11</v>
+      </c>
+      <c r="D87" t="s" s="768">
+        <v>203</v>
+      </c>
+      <c r="E87" t="s" s="769">
+        <v>13</v>
+      </c>
+      <c r="F87" t="s" s="770">
+        <v>14</v>
+      </c>
+      <c r="G87" t="s" s="771">
+        <v>149</v>
+      </c>
+      <c r="H87" t="s" s="772">
+        <v>14</v>
+      </c>
+      <c r="I87" t="s" s="773">
+        <v>17</v>
+      </c>
+      <c r="J87" t="s" s="774">
+        <v>204</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511806" footer="0.511806"/>
   <pageSetup paperSize="1" orientation="portrait" useFirstPageNumber="1"/>

</xml_diff>

<commit_message>
28.07. Aleksa za Vladu
</commit_message>
<xml_diff>
--- a/results/TestResults.xlsx
+++ b/results/TestResults.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>App</t>
   </si>
@@ -57,591 +57,6 @@
   </si>
   <si>
     <t>Description</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Account-Transactions-Filter_By_Type_[WEB]</t>
-  </si>
-  <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:15</t>
-  </si>
-  <si>
-    <t>dev</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>DTC-133</t>
-  </si>
-  <si>
-    <t>Chrome</t>
-  </si>
-  <si>
-    <t>Web</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Account-Transactions-Filter_By_Type_[WEB]_16_06_2026_01_15.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Details-Financial_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:18</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Details-Financial_Details_[WEB]_16_06_2026_01_17.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Details-Account_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:21</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Details-Account_Details_[WEB]_16_06_2026_01_21.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Header-Display_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:23</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Header-Display_[WEB]_16_06_2026_01_23.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions_Filter_By_Date-Date_Picker_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:25</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions_Filter_By_Date-Date_Picker_[WEB]_16_06_2026_01_25.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions-Filter_By_Amount_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:26</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions-Filter_By_Amount_[WEB]_16_06_2026_01_26.jpg</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions_Filter-Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:27</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Accounts-Transactions_Filter-Invalid_[WEB]_16_06_2026_01_27.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments-Back_Button_[WEB]</t>
-  </si>
-  <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:28</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments-Create_New_Recipient_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:31</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments-Create_New_Recipient_[WEB]_16_06_2026_01_31.jpg</t>
-  </si>
-  <si>
-    <t>Domestic_Payments_Modify_Data_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:33</t>
-  </si>
-  <si>
-    <t>Domestic_Payments_In_Future_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:36</t>
-  </si>
-  <si>
-    <t>Domestic_Payments_In_Future_[WEB]_16_06_2026_01_36.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:37</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments-Confirmation_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:41</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments-Confirmation_[WEB]_16_06_2026_01_41.jpg</t>
-  </si>
-  <si>
-    <t>Foreign_Current_Accounts-Transactions-Filter_By_Type_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:42</t>
-  </si>
-  <si>
-    <t>Foreign_Current_Accounts-Transactions-Filter_By_Type_[WEB]_16_06_2026_01_42.jpg</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions_List_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:43</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions_List_[WEB]_16_06_2026_01_43.jpg</t>
-  </si>
-  <si>
-    <t>Foreign_Current_Accounts-Transactions_List_select_Currency_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:46</t>
-  </si>
-  <si>
-    <t>Foreign_Current_Accounts-Transactions_List_select_Currency_[WEB]_16_06_2026_01_46.jpg</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts_Product_Details_Financial_Details_Is_Not_Visible_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:48</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions_List_No_Transactions_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:49</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions_List_No_Transactions_[WEB]_16_06_2026_01_49.jpg</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions-Filter_By_Amount_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:56</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions-Filter_By_Amount_[WEB]_16_06_2026_01_56.jpg</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions-Filter_By_Amount_Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:57</t>
-  </si>
-  <si>
-    <t>Current_Foreign_Accounts-Transactions_Filter-Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:58</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:01:59</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Details_[WEB]_16_06_2026_01_59.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:02</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan_[WEB]_16_06_2026_02_02.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan-Filter_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:05</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan-Filter_[WEB]_16_06_2026_02_05.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan-Filter-invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:07</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan-Filter-invalid_[WEB]_16_06_2026_02_07.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Payments-Filter_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:10</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Payments-Filter_[WEB]_16_06_2026_02_10.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Payments-Filter-invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:12</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Payments-Filter-invalid_[WEB]_16_06_2026_02_12.jpg</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Details-Account_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:15</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Details-Account_Details_[WEB]_16_06_2026_02_15.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-Flow_Disruption_Cancel-Back_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:20</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-Flow_Disruption_Cancel-Back_[WEB]_16_06_2026_02_20.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-From_Current_Account_RSD_[WEB]-To_Current_Account</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:21</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-From_Current_Account_RSD_[WEB]-To_Current_Account_16_06_2026_02_21.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-From_Current_Account_RSD_[WEB]-To_Savings_Account</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:23</t>
-  </si>
-  <si>
-    <t>Payments-Own_Account_Transfer-From_Current_Account_RSD_[WEB]-To_Savings_Account_16_06_2026_02_23.jpg</t>
-  </si>
-  <si>
-    <t>Payments_Payments_Archive-Create_Confirmation_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:24</t>
-  </si>
-  <si>
-    <t>Payments_Payments_Archive-Create_Confirmation_[WEB]_16_06_2026_02_24.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Payments_Overview_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:26</t>
-  </si>
-  <si>
-    <t>Payments-Payments_Overview_[WEB]_16_06_2026_02_26.jpg</t>
-  </si>
-  <si>
-    <t>Product_Summary-Edit_Product_view-edit_name_of_account_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:27</t>
-  </si>
-  <si>
-    <t>Product_Summary-Edit_Product_view-edit_name_of_account_[WEB]_16_06_2026_02_27.jpg</t>
-  </si>
-  <si>
-    <t>Product_Summary-Edit_Product_view-edit_name_of_account-Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:29</t>
-  </si>
-  <si>
-    <t>Product_Summary-Edit_Product_view-edit_name_of_account-Invalid_[WEB]_16_06_2026_02_29.jpg</t>
-  </si>
-  <si>
-    <t>Product_Summary-Hide/Show_Product_on_Product_List_[WEB]_Loan_Accounts</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:30</t>
-  </si>
-  <si>
-    <t>Product_Summary-Hide/Show_Product_on_Product_List_[WEB]_Credit_Cards</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:32</t>
-  </si>
-  <si>
-    <t>Product_Summary-Hide/Show_Product_on_Product_List_[WEB]_Credit_Cards_16_06_2026_02_32.jpg</t>
-  </si>
-  <si>
-    <t>Savings_Accounts-Transactions_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:33</t>
-  </si>
-  <si>
-    <t>Savings_Accounts-Transactions_Details_[WEB]_16_06_2026_02_33.jpg</t>
-  </si>
-  <si>
-    <t>Savings_accounts-Transactions_List_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:35</t>
-  </si>
-  <si>
-    <t>Savings_accounts-Transactions_List_[WEB]_16_06_2026_02_35.jpg</t>
-  </si>
-  <si>
-    <t>Term_Deposits-Details_Account_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:36</t>
-  </si>
-  <si>
-    <t>Term_Deposits-Details_Account_Details_[WEB]_16_06_2026_02_36.jpg</t>
-  </si>
-  <si>
-    <t>Payments-Upcoming_Payments-Cancel_Payments_[WEB]</t>
-  </si>
-  <si>
-    <t>16.06.2026:02:38</t>
-  </si>
-  <si>
-    <t>Payments-Upcoming_Payments-Cancel_Payments_[WEB]_16_06_2026_02_38.jpg</t>
-  </si>
-  <si>
-    <t>16.06.2026:08:38</t>
-  </si>
-  <si>
-    <t>Current_Domestic_Account-Transactions-Filter_By_Type_[WEB]_16_06_2026_08_38.jpg</t>
-  </si>
-  <si>
-    <t>16.06.2026:08:40</t>
-  </si>
-  <si>
-    <t>16.06.2026:08:42</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:03</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:08</t>
-  </si>
-  <si>
-    <t>failed</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:10</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:12</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:19</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Details_[WEB]_16_06_2026_09_19.jpg</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:22</t>
-  </si>
-  <si>
-    <t>Loan_Accounts-Annuity_Plan_[WEB]_16_06_2026_09_22.jpg</t>
-  </si>
-  <si>
-    <t>16.06.2026:09:24</t>
-  </si>
-  <si>
-    <t>Foreign_Current_Account_Product_Details_Account_Details_[WEB]</t>
-  </si>
-  <si>
-    <t>22.07.2026:11:26</t>
-  </si>
-  <si>
-    <t>DTC-103</t>
-  </si>
-  <si>
-    <t>22.07.2026:11:51</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[WEB]</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:29</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:30</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:35</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[WEB]_22_07_2026_13_35.jpg</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:39</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[WEB]_22_07_2026_13_39.jpg</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:44</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[WEB]_22_07_2026_13_44.jpg</t>
-  </si>
-  <si>
-    <t>22.07.2026:13:45</t>
-  </si>
-  <si>
-    <t>22.07.2026:14:12</t>
-  </si>
-  <si>
-    <t>22.07.2026:14:15</t>
-  </si>
-  <si>
-    <t>Payments-Domestic_Payments_[WEB]_22_07_2026_14_15.jpg</t>
-  </si>
-  <si>
-    <t>22.07.2026:14:56</t>
-  </si>
-  <si>
-    <t>23.07.2026:07:04</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:07:23</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]_23_07_2026_07_23.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:07:25</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:07:47</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_23_07_2026_07_47.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:07:55</t>
-  </si>
-  <si>
-    <t>23.07.2026:08:19</t>
-  </si>
-  <si>
-    <t>23.07.2026:08:23</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model11_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:08:32</t>
-  </si>
-  <si>
-    <t>23.07.2026:08:59</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model11_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:02</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:13</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_Invalid_Bez_Poziva_Na_Broj_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:14</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Urgent_Payment_Model97_Invalid_Bez_Poziva_Na_Broj_[WEB]_23_07_2026_09_14.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:15</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model97_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:26</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Purpose_Code_289_Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:32</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:42</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]_23_07_2026_09_42.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:47</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Without_Reference_Number_Invalid_[WEB]_23_07_2026_09_47.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:09:49</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Urgent_Payment_Model97_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:10:03</t>
-  </si>
-  <si>
-    <t>23.07.2026:10:05</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_Budzetski_Non_Urgent_Payment_Model97_[WEB]</t>
-  </si>
-  <si>
-    <t>23.07.2026:10:16</t>
-  </si>
-  <si>
-    <t>23.07.2026:10:18</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model97_[WEB]_23_07_2026_10_18.jpg</t>
-  </si>
-  <si>
-    <t>23.07.2026:10:20</t>
-  </si>
-  <si>
-    <t>Payments_Domestic_Payments_External_Non_Urgent_Payment_Model11_[WEB]_23_07_2026_10_20.jpg</t>
   </si>
 </sst>
 </file>
@@ -813,7 +228,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1010,19 +425,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
@@ -1297,7 +699,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="775">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1307,778 +709,6 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3247,21 +1877,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XFD87"/>
+  <dimension ref="A1:XFD1"/>
   <sheetFormatPr defaultColWidth="8.82407407407407" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="9.33333333333333" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="1" width="39.8611111111111" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="38.2222222222222" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="32.6666666666667" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="28.6666666666667" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="23.2222222222222" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="24.7777777777778" collapsed="true"/>
-    <col min="8" max="9" customWidth="true" style="1" width="28.6666666666667" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="89.5555555555556" collapsed="true"/>
-    <col min="11" max="16372" customWidth="true" style="1" width="8.85185185185185" collapsed="true"/>
-    <col min="16373" max="16373" style="1" width="8.85185185185185" collapsed="true"/>
-    <col min="16374" max="16384" style="1" width="8.82407407407407" collapsed="true"/>
+    <col min="1" max="1" width="9.33333333333333" style="1" customWidth="1"/>
+    <col min="2" max="2" width="39.8611111111111" style="1" customWidth="1"/>
+    <col min="3" max="3" width="38.2222222222222" style="1" customWidth="1"/>
+    <col min="4" max="4" width="32.6666666666667" style="1" customWidth="1"/>
+    <col min="5" max="5" width="28.6666666666667" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.2222222222222" style="1" customWidth="1"/>
+    <col min="7" max="7" width="24.7777777777778" style="1" customWidth="1"/>
+    <col min="8" max="9" width="28.6666666666667" style="1" customWidth="1"/>
+    <col min="10" max="10" width="89.5555555555556" style="1" customWidth="1"/>
+    <col min="11" max="16372" width="8.85185185185185" style="1" customWidth="1"/>
+    <col min="16373" max="16373" width="8.85185185185185" style="1"/>
+    <col min="16374" max="16384" width="8.82407407407407" style="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" ht="13.55" customHeight="1" spans="1:1024 1025:16384">
@@ -19670,2496 +18300,6 @@
       <c r="XFC1" s="1"/>
       <c r="XFD1" s="1"/>
     </row>
-    <row r="2">
-      <c r="B2" t="s" s="3">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s" s="4">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s" s="5">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s" s="6">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s" s="7">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s" s="8">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s" s="9">
-        <v>16</v>
-      </c>
-      <c r="I2" t="s" s="10">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s" s="11">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="s" s="12">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s" s="13">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s" s="14">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s" s="15">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s" s="16">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s" s="17">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s" s="18">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s" s="19">
-        <v>17</v>
-      </c>
-      <c r="J3" t="s" s="20">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="s" s="21">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s" s="22">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s" s="23">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s" s="24">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s" s="25">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s" s="26">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s" s="27">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s" s="28">
-        <v>17</v>
-      </c>
-      <c r="J4" t="s" s="29">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="s" s="30">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s" s="31">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s" s="32">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s" s="33">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s" s="34">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s" s="35">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s" s="36">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s" s="37">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s" s="38">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="s" s="39">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s" s="40">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s" s="41">
-        <v>29</v>
-      </c>
-      <c r="E6" t="s" s="42">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s" s="43">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s" s="44">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s" s="45">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s" s="46">
-        <v>17</v>
-      </c>
-      <c r="J6" t="s" s="47">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="s" s="48">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s" s="49">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s" s="50">
-        <v>32</v>
-      </c>
-      <c r="E7" t="s" s="51">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s" s="52">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s" s="53">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s" s="54">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s" s="55">
-        <v>17</v>
-      </c>
-      <c r="J7" t="s" s="56">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="s" s="57">
-        <v>34</v>
-      </c>
-      <c r="C8" t="s" s="58">
-        <v>11</v>
-      </c>
-      <c r="D8" t="s" s="59">
-        <v>35</v>
-      </c>
-      <c r="E8" t="s" s="60">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s" s="61">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s" s="62">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s" s="63">
-        <v>16</v>
-      </c>
-      <c r="I8" t="s" s="64">
-        <v>17</v>
-      </c>
-      <c r="J8" t="s" s="65">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="s" s="66">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s" s="67">
-        <v>38</v>
-      </c>
-      <c r="D9" t="s" s="68">
-        <v>39</v>
-      </c>
-      <c r="E9" t="s" s="69">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s" s="70">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s" s="71">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s" s="72">
-        <v>16</v>
-      </c>
-      <c r="I9" t="s" s="73">
-        <v>17</v>
-      </c>
-      <c r="J9" t="s" s="74">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="s" s="75">
-        <v>40</v>
-      </c>
-      <c r="C10" t="s" s="76">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s" s="77">
-        <v>41</v>
-      </c>
-      <c r="E10" t="s" s="78">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s" s="79">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s" s="80">
-        <v>15</v>
-      </c>
-      <c r="H10" t="s" s="81">
-        <v>16</v>
-      </c>
-      <c r="I10" t="s" s="82">
-        <v>17</v>
-      </c>
-      <c r="J10" t="s" s="83">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="s" s="84">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s" s="85">
-        <v>38</v>
-      </c>
-      <c r="D11" t="s" s="86">
-        <v>44</v>
-      </c>
-      <c r="E11" t="s" s="87">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s" s="88">
-        <v>14</v>
-      </c>
-      <c r="G11" t="s" s="89">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s" s="90">
-        <v>16</v>
-      </c>
-      <c r="I11" t="s" s="91">
-        <v>17</v>
-      </c>
-      <c r="J11" t="s" s="92">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="s" s="93">
-        <v>45</v>
-      </c>
-      <c r="C12" t="s" s="94">
-        <v>11</v>
-      </c>
-      <c r="D12" t="s" s="95">
-        <v>46</v>
-      </c>
-      <c r="E12" t="s" s="96">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s" s="97">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s" s="98">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s" s="99">
-        <v>16</v>
-      </c>
-      <c r="I12" t="s" s="100">
-        <v>17</v>
-      </c>
-      <c r="J12" t="s" s="101">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="s" s="102">
-        <v>48</v>
-      </c>
-      <c r="C13" t="s" s="103">
-        <v>38</v>
-      </c>
-      <c r="D13" t="s" s="104">
-        <v>49</v>
-      </c>
-      <c r="E13" t="s" s="105">
-        <v>13</v>
-      </c>
-      <c r="F13" t="s" s="106">
-        <v>14</v>
-      </c>
-      <c r="G13" t="s" s="107">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s" s="108">
-        <v>16</v>
-      </c>
-      <c r="I13" t="s" s="109">
-        <v>17</v>
-      </c>
-      <c r="J13" t="s" s="110">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="s" s="111">
-        <v>50</v>
-      </c>
-      <c r="C14" t="s" s="112">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s" s="113">
-        <v>51</v>
-      </c>
-      <c r="E14" t="s" s="114">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s" s="115">
-        <v>14</v>
-      </c>
-      <c r="G14" t="s" s="116">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s" s="117">
-        <v>16</v>
-      </c>
-      <c r="I14" t="s" s="118">
-        <v>17</v>
-      </c>
-      <c r="J14" t="s" s="119">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="s" s="120">
-        <v>53</v>
-      </c>
-      <c r="C15" t="s" s="121">
-        <v>11</v>
-      </c>
-      <c r="D15" t="s" s="122">
-        <v>54</v>
-      </c>
-      <c r="E15" t="s" s="123">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s" s="124">
-        <v>14</v>
-      </c>
-      <c r="G15" t="s" s="125">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s" s="126">
-        <v>16</v>
-      </c>
-      <c r="I15" t="s" s="127">
-        <v>17</v>
-      </c>
-      <c r="J15" t="s" s="128">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="s" s="129">
-        <v>56</v>
-      </c>
-      <c r="C16" t="s" s="130">
-        <v>11</v>
-      </c>
-      <c r="D16" t="s" s="131">
-        <v>57</v>
-      </c>
-      <c r="E16" t="s" s="132">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s" s="133">
-        <v>14</v>
-      </c>
-      <c r="G16" t="s" s="134">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s" s="135">
-        <v>16</v>
-      </c>
-      <c r="I16" t="s" s="136">
-        <v>17</v>
-      </c>
-      <c r="J16" t="s" s="137">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" t="s" s="138">
-        <v>59</v>
-      </c>
-      <c r="C17" t="s" s="139">
-        <v>11</v>
-      </c>
-      <c r="D17" t="s" s="140">
-        <v>60</v>
-      </c>
-      <c r="E17" t="s" s="141">
-        <v>13</v>
-      </c>
-      <c r="F17" t="s" s="142">
-        <v>14</v>
-      </c>
-      <c r="G17" t="s" s="143">
-        <v>15</v>
-      </c>
-      <c r="H17" t="s" s="144">
-        <v>16</v>
-      </c>
-      <c r="I17" t="s" s="145">
-        <v>17</v>
-      </c>
-      <c r="J17" t="s" s="146">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" t="s" s="147">
-        <v>62</v>
-      </c>
-      <c r="C18" t="s" s="148">
-        <v>38</v>
-      </c>
-      <c r="D18" t="s" s="149">
-        <v>63</v>
-      </c>
-      <c r="E18" t="s" s="150">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s" s="151">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s" s="152">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s" s="153">
-        <v>16</v>
-      </c>
-      <c r="I18" t="s" s="154">
-        <v>17</v>
-      </c>
-      <c r="J18" t="s" s="155">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" t="s" s="156">
-        <v>64</v>
-      </c>
-      <c r="C19" t="s" s="157">
-        <v>11</v>
-      </c>
-      <c r="D19" t="s" s="158">
-        <v>65</v>
-      </c>
-      <c r="E19" t="s" s="159">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s" s="160">
-        <v>14</v>
-      </c>
-      <c r="G19" t="s" s="161">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s" s="162">
-        <v>16</v>
-      </c>
-      <c r="I19" t="s" s="163">
-        <v>17</v>
-      </c>
-      <c r="J19" t="s" s="164">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" t="s" s="165">
-        <v>67</v>
-      </c>
-      <c r="C20" t="s" s="166">
-        <v>11</v>
-      </c>
-      <c r="D20" t="s" s="167">
-        <v>68</v>
-      </c>
-      <c r="E20" t="s" s="168">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s" s="169">
-        <v>14</v>
-      </c>
-      <c r="G20" t="s" s="170">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s" s="171">
-        <v>16</v>
-      </c>
-      <c r="I20" t="s" s="172">
-        <v>17</v>
-      </c>
-      <c r="J20" t="s" s="173">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" t="s" s="174">
-        <v>70</v>
-      </c>
-      <c r="C21" t="s" s="175">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s" s="176">
-        <v>71</v>
-      </c>
-      <c r="E21" t="s" s="177">
-        <v>13</v>
-      </c>
-      <c r="F21" t="s" s="178">
-        <v>14</v>
-      </c>
-      <c r="G21" t="s" s="179">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s" s="180">
-        <v>16</v>
-      </c>
-      <c r="I21" t="s" s="181">
-        <v>17</v>
-      </c>
-      <c r="J21" t="s" s="182">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="s" s="183">
-        <v>72</v>
-      </c>
-      <c r="C22" t="s" s="184">
-        <v>38</v>
-      </c>
-      <c r="D22" t="s" s="185">
-        <v>73</v>
-      </c>
-      <c r="E22" t="s" s="186">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s" s="187">
-        <v>14</v>
-      </c>
-      <c r="G22" t="s" s="188">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s" s="189">
-        <v>16</v>
-      </c>
-      <c r="I22" t="s" s="190">
-        <v>17</v>
-      </c>
-      <c r="J22" t="s" s="191">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" t="s" s="192">
-        <v>74</v>
-      </c>
-      <c r="C23" t="s" s="193">
-        <v>11</v>
-      </c>
-      <c r="D23" t="s" s="194">
-        <v>75</v>
-      </c>
-      <c r="E23" t="s" s="195">
-        <v>13</v>
-      </c>
-      <c r="F23" t="s" s="196">
-        <v>14</v>
-      </c>
-      <c r="G23" t="s" s="197">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s" s="198">
-        <v>16</v>
-      </c>
-      <c r="I23" t="s" s="199">
-        <v>17</v>
-      </c>
-      <c r="J23" t="s" s="200">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" t="s" s="201">
-        <v>77</v>
-      </c>
-      <c r="C24" t="s" s="202">
-        <v>11</v>
-      </c>
-      <c r="D24" t="s" s="203">
-        <v>78</v>
-      </c>
-      <c r="E24" t="s" s="204">
-        <v>13</v>
-      </c>
-      <c r="F24" t="s" s="205">
-        <v>14</v>
-      </c>
-      <c r="G24" t="s" s="206">
-        <v>15</v>
-      </c>
-      <c r="H24" t="s" s="207">
-        <v>16</v>
-      </c>
-      <c r="I24" t="s" s="208">
-        <v>17</v>
-      </c>
-      <c r="J24" t="s" s="209">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" t="s" s="210">
-        <v>80</v>
-      </c>
-      <c r="C25" t="s" s="211">
-        <v>11</v>
-      </c>
-      <c r="D25" t="s" s="212">
-        <v>81</v>
-      </c>
-      <c r="E25" t="s" s="213">
-        <v>13</v>
-      </c>
-      <c r="F25" t="s" s="214">
-        <v>14</v>
-      </c>
-      <c r="G25" t="s" s="215">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s" s="216">
-        <v>16</v>
-      </c>
-      <c r="I25" t="s" s="217">
-        <v>17</v>
-      </c>
-      <c r="J25" t="s" s="218">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="s" s="219">
-        <v>83</v>
-      </c>
-      <c r="C26" t="s" s="220">
-        <v>11</v>
-      </c>
-      <c r="D26" t="s" s="221">
-        <v>84</v>
-      </c>
-      <c r="E26" t="s" s="222">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s" s="223">
-        <v>14</v>
-      </c>
-      <c r="G26" t="s" s="224">
-        <v>15</v>
-      </c>
-      <c r="H26" t="s" s="225">
-        <v>16</v>
-      </c>
-      <c r="I26" t="s" s="226">
-        <v>17</v>
-      </c>
-      <c r="J26" t="s" s="227">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="s" s="228">
-        <v>86</v>
-      </c>
-      <c r="C27" t="s" s="229">
-        <v>11</v>
-      </c>
-      <c r="D27" t="s" s="230">
-        <v>87</v>
-      </c>
-      <c r="E27" t="s" s="231">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s" s="232">
-        <v>14</v>
-      </c>
-      <c r="G27" t="s" s="233">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s" s="234">
-        <v>16</v>
-      </c>
-      <c r="I27" t="s" s="235">
-        <v>17</v>
-      </c>
-      <c r="J27" t="s" s="236">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" t="s" s="237">
-        <v>89</v>
-      </c>
-      <c r="C28" t="s" s="238">
-        <v>11</v>
-      </c>
-      <c r="D28" t="s" s="239">
-        <v>90</v>
-      </c>
-      <c r="E28" t="s" s="240">
-        <v>13</v>
-      </c>
-      <c r="F28" t="s" s="241">
-        <v>14</v>
-      </c>
-      <c r="G28" t="s" s="242">
-        <v>15</v>
-      </c>
-      <c r="H28" t="s" s="243">
-        <v>16</v>
-      </c>
-      <c r="I28" t="s" s="244">
-        <v>17</v>
-      </c>
-      <c r="J28" t="s" s="245">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" t="s" s="246">
-        <v>92</v>
-      </c>
-      <c r="C29" t="s" s="247">
-        <v>11</v>
-      </c>
-      <c r="D29" t="s" s="248">
-        <v>93</v>
-      </c>
-      <c r="E29" t="s" s="249">
-        <v>13</v>
-      </c>
-      <c r="F29" t="s" s="250">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s" s="251">
-        <v>15</v>
-      </c>
-      <c r="H29" t="s" s="252">
-        <v>16</v>
-      </c>
-      <c r="I29" t="s" s="253">
-        <v>17</v>
-      </c>
-      <c r="J29" t="s" s="254">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" t="s" s="255">
-        <v>95</v>
-      </c>
-      <c r="C30" t="s" s="256">
-        <v>11</v>
-      </c>
-      <c r="D30" t="s" s="257">
-        <v>96</v>
-      </c>
-      <c r="E30" t="s" s="258">
-        <v>13</v>
-      </c>
-      <c r="F30" t="s" s="259">
-        <v>14</v>
-      </c>
-      <c r="G30" t="s" s="260">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s" s="261">
-        <v>16</v>
-      </c>
-      <c r="I30" t="s" s="262">
-        <v>17</v>
-      </c>
-      <c r="J30" t="s" s="263">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" t="s" s="264">
-        <v>98</v>
-      </c>
-      <c r="C31" t="s" s="265">
-        <v>11</v>
-      </c>
-      <c r="D31" t="s" s="266">
-        <v>99</v>
-      </c>
-      <c r="E31" t="s" s="267">
-        <v>13</v>
-      </c>
-      <c r="F31" t="s" s="268">
-        <v>14</v>
-      </c>
-      <c r="G31" t="s" s="269">
-        <v>15</v>
-      </c>
-      <c r="H31" t="s" s="270">
-        <v>16</v>
-      </c>
-      <c r="I31" t="s" s="271">
-        <v>17</v>
-      </c>
-      <c r="J31" t="s" s="272">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" t="s" s="273">
-        <v>101</v>
-      </c>
-      <c r="C32" t="s" s="274">
-        <v>11</v>
-      </c>
-      <c r="D32" t="s" s="275">
-        <v>102</v>
-      </c>
-      <c r="E32" t="s" s="276">
-        <v>13</v>
-      </c>
-      <c r="F32" t="s" s="277">
-        <v>14</v>
-      </c>
-      <c r="G32" t="s" s="278">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s" s="279">
-        <v>16</v>
-      </c>
-      <c r="I32" t="s" s="280">
-        <v>17</v>
-      </c>
-      <c r="J32" t="s" s="281">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" t="s" s="282">
-        <v>104</v>
-      </c>
-      <c r="C33" t="s" s="283">
-        <v>11</v>
-      </c>
-      <c r="D33" t="s" s="284">
-        <v>105</v>
-      </c>
-      <c r="E33" t="s" s="285">
-        <v>13</v>
-      </c>
-      <c r="F33" t="s" s="286">
-        <v>14</v>
-      </c>
-      <c r="G33" t="s" s="287">
-        <v>15</v>
-      </c>
-      <c r="H33" t="s" s="288">
-        <v>16</v>
-      </c>
-      <c r="I33" t="s" s="289">
-        <v>17</v>
-      </c>
-      <c r="J33" t="s" s="290">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" t="s" s="291">
-        <v>107</v>
-      </c>
-      <c r="C34" t="s" s="292">
-        <v>11</v>
-      </c>
-      <c r="D34" t="s" s="293">
-        <v>108</v>
-      </c>
-      <c r="E34" t="s" s="294">
-        <v>13</v>
-      </c>
-      <c r="F34" t="s" s="295">
-        <v>14</v>
-      </c>
-      <c r="G34" t="s" s="296">
-        <v>15</v>
-      </c>
-      <c r="H34" t="s" s="297">
-        <v>16</v>
-      </c>
-      <c r="I34" t="s" s="298">
-        <v>17</v>
-      </c>
-      <c r="J34" t="s" s="299">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" t="s" s="300">
-        <v>110</v>
-      </c>
-      <c r="C35" t="s" s="301">
-        <v>11</v>
-      </c>
-      <c r="D35" t="s" s="302">
-        <v>111</v>
-      </c>
-      <c r="E35" t="s" s="303">
-        <v>13</v>
-      </c>
-      <c r="F35" t="s" s="304">
-        <v>14</v>
-      </c>
-      <c r="G35" t="s" s="305">
-        <v>15</v>
-      </c>
-      <c r="H35" t="s" s="306">
-        <v>16</v>
-      </c>
-      <c r="I35" t="s" s="307">
-        <v>17</v>
-      </c>
-      <c r="J35" t="s" s="308">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" t="s" s="309">
-        <v>113</v>
-      </c>
-      <c r="C36" t="s" s="310">
-        <v>11</v>
-      </c>
-      <c r="D36" t="s" s="311">
-        <v>114</v>
-      </c>
-      <c r="E36" t="s" s="312">
-        <v>13</v>
-      </c>
-      <c r="F36" t="s" s="313">
-        <v>14</v>
-      </c>
-      <c r="G36" t="s" s="314">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s" s="315">
-        <v>16</v>
-      </c>
-      <c r="I36" t="s" s="316">
-        <v>17</v>
-      </c>
-      <c r="J36" t="s" s="317">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" t="s" s="318">
-        <v>116</v>
-      </c>
-      <c r="C37" t="s" s="319">
-        <v>38</v>
-      </c>
-      <c r="D37" t="s" s="320">
-        <v>117</v>
-      </c>
-      <c r="E37" t="s" s="321">
-        <v>13</v>
-      </c>
-      <c r="F37" t="s" s="322">
-        <v>14</v>
-      </c>
-      <c r="G37" t="s" s="323">
-        <v>15</v>
-      </c>
-      <c r="H37" t="s" s="324">
-        <v>16</v>
-      </c>
-      <c r="I37" t="s" s="325">
-        <v>17</v>
-      </c>
-      <c r="J37" t="s" s="326">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" t="s" s="327">
-        <v>118</v>
-      </c>
-      <c r="C38" t="s" s="328">
-        <v>11</v>
-      </c>
-      <c r="D38" t="s" s="329">
-        <v>119</v>
-      </c>
-      <c r="E38" t="s" s="330">
-        <v>13</v>
-      </c>
-      <c r="F38" t="s" s="331">
-        <v>14</v>
-      </c>
-      <c r="G38" t="s" s="332">
-        <v>15</v>
-      </c>
-      <c r="H38" t="s" s="333">
-        <v>16</v>
-      </c>
-      <c r="I38" t="s" s="334">
-        <v>17</v>
-      </c>
-      <c r="J38" t="s" s="335">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" t="s" s="336">
-        <v>121</v>
-      </c>
-      <c r="C39" t="s" s="337">
-        <v>11</v>
-      </c>
-      <c r="D39" t="s" s="338">
-        <v>122</v>
-      </c>
-      <c r="E39" t="s" s="339">
-        <v>13</v>
-      </c>
-      <c r="F39" t="s" s="340">
-        <v>14</v>
-      </c>
-      <c r="G39" t="s" s="341">
-        <v>15</v>
-      </c>
-      <c r="H39" t="s" s="342">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s" s="343">
-        <v>17</v>
-      </c>
-      <c r="J39" t="s" s="344">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" t="s" s="345">
-        <v>124</v>
-      </c>
-      <c r="C40" t="s" s="346">
-        <v>11</v>
-      </c>
-      <c r="D40" t="s" s="347">
-        <v>125</v>
-      </c>
-      <c r="E40" t="s" s="348">
-        <v>13</v>
-      </c>
-      <c r="F40" t="s" s="349">
-        <v>14</v>
-      </c>
-      <c r="G40" t="s" s="350">
-        <v>15</v>
-      </c>
-      <c r="H40" t="s" s="351">
-        <v>16</v>
-      </c>
-      <c r="I40" t="s" s="352">
-        <v>17</v>
-      </c>
-      <c r="J40" t="s" s="353">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" t="s" s="354">
-        <v>127</v>
-      </c>
-      <c r="C41" t="s" s="355">
-        <v>11</v>
-      </c>
-      <c r="D41" t="s" s="356">
-        <v>128</v>
-      </c>
-      <c r="E41" t="s" s="357">
-        <v>13</v>
-      </c>
-      <c r="F41" t="s" s="358">
-        <v>14</v>
-      </c>
-      <c r="G41" t="s" s="359">
-        <v>15</v>
-      </c>
-      <c r="H41" t="s" s="360">
-        <v>16</v>
-      </c>
-      <c r="I41" t="s" s="361">
-        <v>17</v>
-      </c>
-      <c r="J41" t="s" s="362">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" t="s" s="363">
-        <v>130</v>
-      </c>
-      <c r="C42" t="s" s="364">
-        <v>11</v>
-      </c>
-      <c r="D42" t="s" s="365">
-        <v>131</v>
-      </c>
-      <c r="E42" t="s" s="366">
-        <v>13</v>
-      </c>
-      <c r="F42" t="s" s="367">
-        <v>14</v>
-      </c>
-      <c r="G42" t="s" s="368">
-        <v>15</v>
-      </c>
-      <c r="H42" t="s" s="369">
-        <v>16</v>
-      </c>
-      <c r="I42" t="s" s="370">
-        <v>17</v>
-      </c>
-      <c r="J42" t="s" s="371">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" t="s" s="372">
-        <v>10</v>
-      </c>
-      <c r="C43" t="s" s="373">
-        <v>11</v>
-      </c>
-      <c r="D43" t="s" s="374">
-        <v>133</v>
-      </c>
-      <c r="E43" t="s" s="375">
-        <v>13</v>
-      </c>
-      <c r="F43" t="s" s="376">
-        <v>14</v>
-      </c>
-      <c r="G43" t="s" s="377">
-        <v>15</v>
-      </c>
-      <c r="H43" t="s" s="378">
-        <v>14</v>
-      </c>
-      <c r="I43" t="s" s="379">
-        <v>17</v>
-      </c>
-      <c r="J43" t="s" s="380">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" t="s" s="381">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s" s="382">
-        <v>38</v>
-      </c>
-      <c r="D44" t="s" s="383">
-        <v>135</v>
-      </c>
-      <c r="E44" t="s" s="384">
-        <v>13</v>
-      </c>
-      <c r="F44" t="s" s="385">
-        <v>14</v>
-      </c>
-      <c r="G44" t="s" s="386">
-        <v>15</v>
-      </c>
-      <c r="H44" t="s" s="387">
-        <v>14</v>
-      </c>
-      <c r="I44" t="s" s="388">
-        <v>17</v>
-      </c>
-      <c r="J44" t="s" s="389">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" t="s" s="390">
-        <v>110</v>
-      </c>
-      <c r="C45" t="s" s="391">
-        <v>38</v>
-      </c>
-      <c r="D45" t="s" s="392">
-        <v>136</v>
-      </c>
-      <c r="E45" t="s" s="393">
-        <v>13</v>
-      </c>
-      <c r="F45" t="s" s="394">
-        <v>14</v>
-      </c>
-      <c r="G45" t="s" s="395">
-        <v>15</v>
-      </c>
-      <c r="H45" t="s" s="396">
-        <v>14</v>
-      </c>
-      <c r="I45" t="s" s="397">
-        <v>17</v>
-      </c>
-      <c r="J45" t="s" s="398">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" t="s" s="399">
-        <v>113</v>
-      </c>
-      <c r="C46" t="s" s="400">
-        <v>38</v>
-      </c>
-      <c r="D46" t="s" s="401">
-        <v>137</v>
-      </c>
-      <c r="E46" t="s" s="402">
-        <v>13</v>
-      </c>
-      <c r="F46" t="s" s="403">
-        <v>14</v>
-      </c>
-      <c r="G46" t="s" s="404">
-        <v>15</v>
-      </c>
-      <c r="H46" t="s" s="405">
-        <v>14</v>
-      </c>
-      <c r="I46" t="s" s="406">
-        <v>17</v>
-      </c>
-      <c r="J46" t="s" s="407">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" t="s" s="408">
-        <v>40</v>
-      </c>
-      <c r="C47" t="s" s="409">
-        <v>11</v>
-      </c>
-      <c r="D47" t="s" s="410">
-        <v>138</v>
-      </c>
-      <c r="E47" t="s" s="411">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s" s="412">
-        <v>14</v>
-      </c>
-      <c r="G47" t="s" s="413">
-        <v>15</v>
-      </c>
-      <c r="H47" t="s" s="414">
-        <v>14</v>
-      </c>
-      <c r="I47" t="s" s="415">
-        <v>17</v>
-      </c>
-      <c r="J47" t="s" s="416">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" t="s" s="417">
-        <v>43</v>
-      </c>
-      <c r="C48" t="s" s="418">
-        <v>11</v>
-      </c>
-      <c r="D48" t="s" s="419">
-        <v>140</v>
-      </c>
-      <c r="E48" t="s" s="420">
-        <v>13</v>
-      </c>
-      <c r="F48" t="s" s="421">
-        <v>14</v>
-      </c>
-      <c r="G48" t="s" s="422">
-        <v>15</v>
-      </c>
-      <c r="H48" t="s" s="423">
-        <v>14</v>
-      </c>
-      <c r="I48" t="s" s="424">
-        <v>17</v>
-      </c>
-      <c r="J48" t="s" s="425">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" t="s" s="426">
-        <v>43</v>
-      </c>
-      <c r="C49" t="s" s="427">
-        <v>11</v>
-      </c>
-      <c r="D49" t="s" s="428">
-        <v>141</v>
-      </c>
-      <c r="E49" t="s" s="429">
-        <v>13</v>
-      </c>
-      <c r="F49" t="s" s="430">
-        <v>14</v>
-      </c>
-      <c r="G49" t="s" s="431">
-        <v>15</v>
-      </c>
-      <c r="H49" t="s" s="432">
-        <v>14</v>
-      </c>
-      <c r="I49" t="s" s="433">
-        <v>17</v>
-      </c>
-      <c r="J49" t="s" s="434">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" t="s" s="435">
-        <v>74</v>
-      </c>
-      <c r="C50" t="s" s="436">
-        <v>11</v>
-      </c>
-      <c r="D50" t="s" s="437">
-        <v>142</v>
-      </c>
-      <c r="E50" t="s" s="438">
-        <v>13</v>
-      </c>
-      <c r="F50" t="s" s="439">
-        <v>14</v>
-      </c>
-      <c r="G50" t="s" s="440">
-        <v>15</v>
-      </c>
-      <c r="H50" t="s" s="441">
-        <v>14</v>
-      </c>
-      <c r="I50" t="s" s="442">
-        <v>17</v>
-      </c>
-      <c r="J50" t="s" s="443">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" t="s" s="444">
-        <v>77</v>
-      </c>
-      <c r="C51" t="s" s="445">
-        <v>11</v>
-      </c>
-      <c r="D51" t="s" s="446">
-        <v>144</v>
-      </c>
-      <c r="E51" t="s" s="447">
-        <v>13</v>
-      </c>
-      <c r="F51" t="s" s="448">
-        <v>14</v>
-      </c>
-      <c r="G51" t="s" s="449">
-        <v>15</v>
-      </c>
-      <c r="H51" t="s" s="450">
-        <v>14</v>
-      </c>
-      <c r="I51" t="s" s="451">
-        <v>17</v>
-      </c>
-      <c r="J51" t="s" s="452">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" t="s" s="453">
-        <v>77</v>
-      </c>
-      <c r="C52" t="s" s="454">
-        <v>38</v>
-      </c>
-      <c r="D52" t="s" s="455">
-        <v>146</v>
-      </c>
-      <c r="E52" t="s" s="456">
-        <v>13</v>
-      </c>
-      <c r="F52" t="s" s="457">
-        <v>14</v>
-      </c>
-      <c r="G52" t="s" s="458">
-        <v>15</v>
-      </c>
-      <c r="H52" t="s" s="459">
-        <v>14</v>
-      </c>
-      <c r="I52" t="s" s="460">
-        <v>17</v>
-      </c>
-      <c r="J52" t="s" s="461">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" t="s" s="462">
-        <v>147</v>
-      </c>
-      <c r="C53" t="s" s="463">
-        <v>11</v>
-      </c>
-      <c r="D53" t="s" s="464">
-        <v>148</v>
-      </c>
-      <c r="E53" t="s" s="465">
-        <v>13</v>
-      </c>
-      <c r="F53" t="s" s="466">
-        <v>14</v>
-      </c>
-      <c r="G53" t="s" s="467">
-        <v>149</v>
-      </c>
-      <c r="H53" t="s" s="468">
-        <v>14</v>
-      </c>
-      <c r="I53" t="s" s="469">
-        <v>17</v>
-      </c>
-      <c r="J53" t="s" s="470">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" t="s" s="471">
-        <v>147</v>
-      </c>
-      <c r="C54" t="s" s="472">
-        <v>11</v>
-      </c>
-      <c r="D54" t="s" s="473">
-        <v>150</v>
-      </c>
-      <c r="E54" t="s" s="474">
-        <v>13</v>
-      </c>
-      <c r="F54" t="s" s="475">
-        <v>14</v>
-      </c>
-      <c r="G54" t="s" s="476">
-        <v>149</v>
-      </c>
-      <c r="H54" t="s" s="477">
-        <v>14</v>
-      </c>
-      <c r="I54" t="s" s="478">
-        <v>17</v>
-      </c>
-      <c r="J54" t="s" s="479">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" t="s" s="480">
-        <v>151</v>
-      </c>
-      <c r="C55" t="s" s="481">
-        <v>11</v>
-      </c>
-      <c r="D55" t="s" s="482">
-        <v>152</v>
-      </c>
-      <c r="E55" t="s" s="483">
-        <v>13</v>
-      </c>
-      <c r="F55" t="s" s="484">
-        <v>14</v>
-      </c>
-      <c r="G55" t="s" s="485">
-        <v>149</v>
-      </c>
-      <c r="H55" t="s" s="486">
-        <v>14</v>
-      </c>
-      <c r="I55" t="s" s="487">
-        <v>17</v>
-      </c>
-      <c r="J55" t="s" s="488">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" t="s" s="489">
-        <v>151</v>
-      </c>
-      <c r="C56" t="s" s="490">
-        <v>11</v>
-      </c>
-      <c r="D56" t="s" s="491">
-        <v>153</v>
-      </c>
-      <c r="E56" t="s" s="492">
-        <v>13</v>
-      </c>
-      <c r="F56" t="s" s="493">
-        <v>14</v>
-      </c>
-      <c r="G56" t="s" s="494">
-        <v>149</v>
-      </c>
-      <c r="H56" t="s" s="495">
-        <v>14</v>
-      </c>
-      <c r="I56" t="s" s="496">
-        <v>17</v>
-      </c>
-      <c r="J56" t="s" s="497">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" t="s" s="498">
-        <v>151</v>
-      </c>
-      <c r="C57" t="s" s="499">
-        <v>11</v>
-      </c>
-      <c r="D57" t="s" s="500">
-        <v>154</v>
-      </c>
-      <c r="E57" t="s" s="501">
-        <v>13</v>
-      </c>
-      <c r="F57" t="s" s="502">
-        <v>14</v>
-      </c>
-      <c r="G57" t="s" s="503">
-        <v>149</v>
-      </c>
-      <c r="H57" t="s" s="504">
-        <v>14</v>
-      </c>
-      <c r="I57" t="s" s="505">
-        <v>17</v>
-      </c>
-      <c r="J57" t="s" s="506">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" t="s" s="507">
-        <v>151</v>
-      </c>
-      <c r="C58" t="s" s="508">
-        <v>11</v>
-      </c>
-      <c r="D58" t="s" s="509">
-        <v>156</v>
-      </c>
-      <c r="E58"/>
-      <c r="F58" t="s" s="510">
-        <v>14</v>
-      </c>
-      <c r="G58" t="s" s="511">
-        <v>149</v>
-      </c>
-      <c r="H58" t="s" s="512">
-        <v>14</v>
-      </c>
-      <c r="I58" t="s" s="513">
-        <v>17</v>
-      </c>
-      <c r="J58" t="s" s="514">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" t="s" s="515">
-        <v>151</v>
-      </c>
-      <c r="C59" t="s" s="516">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s" s="517">
-        <v>156</v>
-      </c>
-      <c r="E59"/>
-      <c r="F59" t="s" s="518">
-        <v>14</v>
-      </c>
-      <c r="G59" t="s" s="519">
-        <v>149</v>
-      </c>
-      <c r="H59" t="s" s="520">
-        <v>14</v>
-      </c>
-      <c r="I59" t="s" s="521">
-        <v>17</v>
-      </c>
-      <c r="J59" t="s" s="522">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" t="s" s="523">
-        <v>151</v>
-      </c>
-      <c r="C60" t="s" s="524">
-        <v>11</v>
-      </c>
-      <c r="D60" t="s" s="525">
-        <v>158</v>
-      </c>
-      <c r="E60" t="s" s="526">
-        <v>13</v>
-      </c>
-      <c r="F60" t="s" s="527">
-        <v>14</v>
-      </c>
-      <c r="G60" t="s" s="528">
-        <v>149</v>
-      </c>
-      <c r="H60" t="s" s="529">
-        <v>14</v>
-      </c>
-      <c r="I60" t="s" s="530">
-        <v>17</v>
-      </c>
-      <c r="J60" t="s" s="531">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" t="s" s="532">
-        <v>151</v>
-      </c>
-      <c r="C61" t="s" s="533">
-        <v>38</v>
-      </c>
-      <c r="D61" t="s" s="534">
-        <v>160</v>
-      </c>
-      <c r="E61" t="s" s="535">
-        <v>13</v>
-      </c>
-      <c r="F61" t="s" s="536">
-        <v>14</v>
-      </c>
-      <c r="G61" t="s" s="537">
-        <v>149</v>
-      </c>
-      <c r="H61" t="s" s="538">
-        <v>14</v>
-      </c>
-      <c r="I61" t="s" s="539">
-        <v>17</v>
-      </c>
-      <c r="J61" t="s" s="540">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" t="s" s="541">
-        <v>151</v>
-      </c>
-      <c r="C62" t="s" s="542">
-        <v>38</v>
-      </c>
-      <c r="D62" t="s" s="543">
-        <v>161</v>
-      </c>
-      <c r="E62" t="s" s="544">
-        <v>13</v>
-      </c>
-      <c r="F62" t="s" s="545">
-        <v>14</v>
-      </c>
-      <c r="G62" t="s" s="546">
-        <v>149</v>
-      </c>
-      <c r="H62" t="s" s="547">
-        <v>14</v>
-      </c>
-      <c r="I62" t="s" s="548">
-        <v>17</v>
-      </c>
-      <c r="J62" t="s" s="549">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" t="s" s="550">
-        <v>48</v>
-      </c>
-      <c r="C63" t="s" s="551">
-        <v>11</v>
-      </c>
-      <c r="D63" t="s" s="552">
-        <v>162</v>
-      </c>
-      <c r="E63" t="s" s="553">
-        <v>13</v>
-      </c>
-      <c r="F63" t="s" s="554">
-        <v>14</v>
-      </c>
-      <c r="G63" t="s" s="555">
-        <v>149</v>
-      </c>
-      <c r="H63" t="s" s="556">
-        <v>14</v>
-      </c>
-      <c r="I63" t="s" s="557">
-        <v>17</v>
-      </c>
-      <c r="J63" t="s" s="558">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" t="s" s="559">
-        <v>151</v>
-      </c>
-      <c r="C64" t="s" s="560">
-        <v>38</v>
-      </c>
-      <c r="D64" t="s" s="561">
-        <v>164</v>
-      </c>
-      <c r="E64" t="s" s="562">
-        <v>13</v>
-      </c>
-      <c r="F64" t="s" s="563">
-        <v>14</v>
-      </c>
-      <c r="G64" t="s" s="564">
-        <v>149</v>
-      </c>
-      <c r="H64" t="s" s="565">
-        <v>14</v>
-      </c>
-      <c r="I64" t="s" s="566">
-        <v>17</v>
-      </c>
-      <c r="J64" t="s" s="567">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" t="s" s="568">
-        <v>151</v>
-      </c>
-      <c r="C65" t="s" s="569">
-        <v>38</v>
-      </c>
-      <c r="D65" t="s" s="570">
-        <v>165</v>
-      </c>
-      <c r="E65" t="s" s="571">
-        <v>13</v>
-      </c>
-      <c r="F65" t="s" s="572">
-        <v>14</v>
-      </c>
-      <c r="G65" t="s" s="573">
-        <v>149</v>
-      </c>
-      <c r="H65" t="s" s="574">
-        <v>14</v>
-      </c>
-      <c r="I65" t="s" s="575">
-        <v>17</v>
-      </c>
-      <c r="J65" t="s" s="576">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" t="s" s="577">
-        <v>166</v>
-      </c>
-      <c r="C66" t="s" s="578">
-        <v>11</v>
-      </c>
-      <c r="D66" t="s" s="579">
-        <v>167</v>
-      </c>
-      <c r="E66" t="s" s="580">
-        <v>13</v>
-      </c>
-      <c r="F66" t="s" s="581">
-        <v>14</v>
-      </c>
-      <c r="G66" t="s" s="582">
-        <v>149</v>
-      </c>
-      <c r="H66" t="s" s="583">
-        <v>14</v>
-      </c>
-      <c r="I66" t="s" s="584">
-        <v>17</v>
-      </c>
-      <c r="J66" t="s" s="585">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" t="s" s="586">
-        <v>166</v>
-      </c>
-      <c r="C67" t="s" s="587">
-        <v>38</v>
-      </c>
-      <c r="D67" t="s" s="588">
-        <v>169</v>
-      </c>
-      <c r="E67" t="s" s="589">
-        <v>13</v>
-      </c>
-      <c r="F67" t="s" s="590">
-        <v>14</v>
-      </c>
-      <c r="G67" t="s" s="591">
-        <v>149</v>
-      </c>
-      <c r="H67" t="s" s="592">
-        <v>14</v>
-      </c>
-      <c r="I67" t="s" s="593">
-        <v>17</v>
-      </c>
-      <c r="J67" t="s" s="594">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" t="s" s="595">
-        <v>170</v>
-      </c>
-      <c r="C68" t="s" s="596">
-        <v>11</v>
-      </c>
-      <c r="D68" t="s" s="597">
-        <v>171</v>
-      </c>
-      <c r="E68" t="s" s="598">
-        <v>13</v>
-      </c>
-      <c r="F68" t="s" s="599">
-        <v>14</v>
-      </c>
-      <c r="G68" t="s" s="600">
-        <v>149</v>
-      </c>
-      <c r="H68" t="s" s="601">
-        <v>14</v>
-      </c>
-      <c r="I68" t="s" s="602">
-        <v>17</v>
-      </c>
-      <c r="J68" t="s" s="603">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" t="s" s="604">
-        <v>170</v>
-      </c>
-      <c r="C69" t="s" s="605">
-        <v>38</v>
-      </c>
-      <c r="D69" t="s" s="606">
-        <v>173</v>
-      </c>
-      <c r="E69" t="s" s="607">
-        <v>13</v>
-      </c>
-      <c r="F69" t="s" s="608">
-        <v>14</v>
-      </c>
-      <c r="G69" t="s" s="609">
-        <v>149</v>
-      </c>
-      <c r="H69" t="s" s="610">
-        <v>14</v>
-      </c>
-      <c r="I69" t="s" s="611">
-        <v>17</v>
-      </c>
-      <c r="J69" t="s" s="612">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" t="s" s="613">
-        <v>170</v>
-      </c>
-      <c r="C70" t="s" s="614">
-        <v>38</v>
-      </c>
-      <c r="D70" t="s" s="615">
-        <v>174</v>
-      </c>
-      <c r="E70" t="s" s="616">
-        <v>13</v>
-      </c>
-      <c r="F70" t="s" s="617">
-        <v>14</v>
-      </c>
-      <c r="G70" t="s" s="618">
-        <v>149</v>
-      </c>
-      <c r="H70" t="s" s="619">
-        <v>14</v>
-      </c>
-      <c r="I70" t="s" s="620">
-        <v>17</v>
-      </c>
-      <c r="J70" t="s" s="621">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" t="s" s="622">
-        <v>166</v>
-      </c>
-      <c r="C71" t="s" s="623">
-        <v>38</v>
-      </c>
-      <c r="D71" t="s" s="624">
-        <v>175</v>
-      </c>
-      <c r="E71" t="s" s="625">
-        <v>13</v>
-      </c>
-      <c r="F71" t="s" s="626">
-        <v>14</v>
-      </c>
-      <c r="G71" t="s" s="627">
-        <v>149</v>
-      </c>
-      <c r="H71" t="s" s="628">
-        <v>14</v>
-      </c>
-      <c r="I71" t="s" s="629">
-        <v>17</v>
-      </c>
-      <c r="J71" t="s" s="630">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="s" s="631">
-        <v>176</v>
-      </c>
-      <c r="C72" t="s" s="632">
-        <v>38</v>
-      </c>
-      <c r="D72" t="s" s="633">
-        <v>177</v>
-      </c>
-      <c r="E72" t="s" s="634">
-        <v>13</v>
-      </c>
-      <c r="F72" t="s" s="635">
-        <v>14</v>
-      </c>
-      <c r="G72" t="s" s="636">
-        <v>149</v>
-      </c>
-      <c r="H72" t="s" s="637">
-        <v>14</v>
-      </c>
-      <c r="I72" t="s" s="638">
-        <v>17</v>
-      </c>
-      <c r="J72" t="s" s="639">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="s" s="640">
-        <v>176</v>
-      </c>
-      <c r="C73" t="s" s="641">
-        <v>38</v>
-      </c>
-      <c r="D73" t="s" s="642">
-        <v>178</v>
-      </c>
-      <c r="E73" t="s" s="643">
-        <v>13</v>
-      </c>
-      <c r="F73" t="s" s="644">
-        <v>14</v>
-      </c>
-      <c r="G73" t="s" s="645">
-        <v>149</v>
-      </c>
-      <c r="H73" t="s" s="646">
-        <v>14</v>
-      </c>
-      <c r="I73" t="s" s="647">
-        <v>17</v>
-      </c>
-      <c r="J73" t="s" s="648">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" t="s" s="649">
-        <v>179</v>
-      </c>
-      <c r="C74" t="s" s="650">
-        <v>38</v>
-      </c>
-      <c r="D74" t="s" s="651">
-        <v>180</v>
-      </c>
-      <c r="E74" t="s" s="652">
-        <v>13</v>
-      </c>
-      <c r="F74" t="s" s="653">
-        <v>14</v>
-      </c>
-      <c r="G74" t="s" s="654">
-        <v>149</v>
-      </c>
-      <c r="H74" t="s" s="655">
-        <v>14</v>
-      </c>
-      <c r="I74" t="s" s="656">
-        <v>17</v>
-      </c>
-      <c r="J74" t="s" s="657">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" t="s" s="658">
-        <v>176</v>
-      </c>
-      <c r="C75" t="s" s="659">
-        <v>38</v>
-      </c>
-      <c r="D75" t="s" s="660">
-        <v>181</v>
-      </c>
-      <c r="E75" t="s" s="661">
-        <v>13</v>
-      </c>
-      <c r="F75" t="s" s="662">
-        <v>14</v>
-      </c>
-      <c r="G75" t="s" s="663">
-        <v>149</v>
-      </c>
-      <c r="H75" t="s" s="664">
-        <v>14</v>
-      </c>
-      <c r="I75" t="s" s="665">
-        <v>17</v>
-      </c>
-      <c r="J75" t="s" s="666">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" t="s" s="667">
-        <v>182</v>
-      </c>
-      <c r="C76" t="s" s="668">
-        <v>11</v>
-      </c>
-      <c r="D76" t="s" s="669">
-        <v>183</v>
-      </c>
-      <c r="E76" t="s" s="670">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s" s="671">
-        <v>14</v>
-      </c>
-      <c r="G76" t="s" s="672">
-        <v>149</v>
-      </c>
-      <c r="H76" t="s" s="673">
-        <v>14</v>
-      </c>
-      <c r="I76" t="s" s="674">
-        <v>17</v>
-      </c>
-      <c r="J76" t="s" s="675">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" t="s" s="676">
-        <v>182</v>
-      </c>
-      <c r="C77" t="s" s="677">
-        <v>38</v>
-      </c>
-      <c r="D77" t="s" s="678">
-        <v>185</v>
-      </c>
-      <c r="E77" t="s" s="679">
-        <v>13</v>
-      </c>
-      <c r="F77" t="s" s="680">
-        <v>14</v>
-      </c>
-      <c r="G77" t="s" s="681">
-        <v>149</v>
-      </c>
-      <c r="H77" t="s" s="682">
-        <v>14</v>
-      </c>
-      <c r="I77" t="s" s="683">
-        <v>17</v>
-      </c>
-      <c r="J77" t="s" s="684">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" t="s" s="685">
-        <v>186</v>
-      </c>
-      <c r="C78" t="s" s="686">
-        <v>38</v>
-      </c>
-      <c r="D78" t="s" s="687">
-        <v>187</v>
-      </c>
-      <c r="E78" t="s" s="688">
-        <v>13</v>
-      </c>
-      <c r="F78" t="s" s="689">
-        <v>14</v>
-      </c>
-      <c r="G78" t="s" s="690">
-        <v>149</v>
-      </c>
-      <c r="H78" t="s" s="691">
-        <v>14</v>
-      </c>
-      <c r="I78" t="s" s="692">
-        <v>17</v>
-      </c>
-      <c r="J78" t="s" s="693">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" t="s" s="694">
-        <v>188</v>
-      </c>
-      <c r="C79" t="s" s="695">
-        <v>38</v>
-      </c>
-      <c r="D79" t="s" s="696">
-        <v>189</v>
-      </c>
-      <c r="E79" t="s" s="697">
-        <v>13</v>
-      </c>
-      <c r="F79" t="s" s="698">
-        <v>14</v>
-      </c>
-      <c r="G79" t="s" s="699">
-        <v>149</v>
-      </c>
-      <c r="H79" t="s" s="700">
-        <v>14</v>
-      </c>
-      <c r="I79" t="s" s="701">
-        <v>17</v>
-      </c>
-      <c r="J79" t="s" s="702">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" t="s" s="703">
-        <v>190</v>
-      </c>
-      <c r="C80" t="s" s="704">
-        <v>11</v>
-      </c>
-      <c r="D80" t="s" s="705">
-        <v>191</v>
-      </c>
-      <c r="E80" t="s" s="706">
-        <v>13</v>
-      </c>
-      <c r="F80" t="s" s="707">
-        <v>14</v>
-      </c>
-      <c r="G80" t="s" s="708">
-        <v>149</v>
-      </c>
-      <c r="H80" t="s" s="709">
-        <v>14</v>
-      </c>
-      <c r="I80" t="s" s="710">
-        <v>17</v>
-      </c>
-      <c r="J80" t="s" s="711">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" t="s" s="712">
-        <v>190</v>
-      </c>
-      <c r="C81" t="s" s="713">
-        <v>11</v>
-      </c>
-      <c r="D81" t="s" s="714">
-        <v>193</v>
-      </c>
-      <c r="E81" t="s" s="715">
-        <v>13</v>
-      </c>
-      <c r="F81" t="s" s="716">
-        <v>14</v>
-      </c>
-      <c r="G81" t="s" s="717">
-        <v>149</v>
-      </c>
-      <c r="H81" t="s" s="718">
-        <v>14</v>
-      </c>
-      <c r="I81" t="s" s="719">
-        <v>17</v>
-      </c>
-      <c r="J81" t="s" s="720">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" t="s" s="721">
-        <v>190</v>
-      </c>
-      <c r="C82" t="s" s="722">
-        <v>38</v>
-      </c>
-      <c r="D82" t="s" s="723">
-        <v>195</v>
-      </c>
-      <c r="E82" t="s" s="724">
-        <v>13</v>
-      </c>
-      <c r="F82" t="s" s="725">
-        <v>14</v>
-      </c>
-      <c r="G82" t="s" s="726">
-        <v>149</v>
-      </c>
-      <c r="H82" t="s" s="727">
-        <v>14</v>
-      </c>
-      <c r="I82" t="s" s="728">
-        <v>17</v>
-      </c>
-      <c r="J82" t="s" s="729">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" t="s" s="730">
-        <v>196</v>
-      </c>
-      <c r="C83" t="s" s="731">
-        <v>38</v>
-      </c>
-      <c r="D83" t="s" s="732">
-        <v>197</v>
-      </c>
-      <c r="E83" t="s" s="733">
-        <v>13</v>
-      </c>
-      <c r="F83" t="s" s="734">
-        <v>14</v>
-      </c>
-      <c r="G83" t="s" s="735">
-        <v>149</v>
-      </c>
-      <c r="H83" t="s" s="736">
-        <v>14</v>
-      </c>
-      <c r="I83" t="s" s="737">
-        <v>17</v>
-      </c>
-      <c r="J83" t="s" s="738">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" t="s" s="739">
-        <v>196</v>
-      </c>
-      <c r="C84" t="s" s="740">
-        <v>38</v>
-      </c>
-      <c r="D84" t="s" s="741">
-        <v>198</v>
-      </c>
-      <c r="E84" t="s" s="742">
-        <v>13</v>
-      </c>
-      <c r="F84" t="s" s="743">
-        <v>14</v>
-      </c>
-      <c r="G84" t="s" s="744">
-        <v>149</v>
-      </c>
-      <c r="H84" t="s" s="745">
-        <v>14</v>
-      </c>
-      <c r="I84" t="s" s="746">
-        <v>17</v>
-      </c>
-      <c r="J84" t="s" s="747">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" t="s" s="748">
-        <v>199</v>
-      </c>
-      <c r="C85" t="s" s="749">
-        <v>38</v>
-      </c>
-      <c r="D85" t="s" s="750">
-        <v>200</v>
-      </c>
-      <c r="E85" t="s" s="751">
-        <v>13</v>
-      </c>
-      <c r="F85" t="s" s="752">
-        <v>14</v>
-      </c>
-      <c r="G85" t="s" s="753">
-        <v>149</v>
-      </c>
-      <c r="H85" t="s" s="754">
-        <v>14</v>
-      </c>
-      <c r="I85" t="s" s="755">
-        <v>17</v>
-      </c>
-      <c r="J85" t="s" s="756">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" t="s" s="757">
-        <v>186</v>
-      </c>
-      <c r="C86" t="s" s="758">
-        <v>11</v>
-      </c>
-      <c r="D86" t="s" s="759">
-        <v>201</v>
-      </c>
-      <c r="E86" t="s" s="760">
-        <v>13</v>
-      </c>
-      <c r="F86" t="s" s="761">
-        <v>14</v>
-      </c>
-      <c r="G86" t="s" s="762">
-        <v>149</v>
-      </c>
-      <c r="H86" t="s" s="763">
-        <v>14</v>
-      </c>
-      <c r="I86" t="s" s="764">
-        <v>17</v>
-      </c>
-      <c r="J86" t="s" s="765">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" t="s" s="766">
-        <v>179</v>
-      </c>
-      <c r="C87" t="s" s="767">
-        <v>11</v>
-      </c>
-      <c r="D87" t="s" s="768">
-        <v>203</v>
-      </c>
-      <c r="E87" t="s" s="769">
-        <v>13</v>
-      </c>
-      <c r="F87" t="s" s="770">
-        <v>14</v>
-      </c>
-      <c r="G87" t="s" s="771">
-        <v>149</v>
-      </c>
-      <c r="H87" t="s" s="772">
-        <v>14</v>
-      </c>
-      <c r="I87" t="s" s="773">
-        <v>17</v>
-      </c>
-      <c r="J87" t="s" s="774">
-        <v>204</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511806" footer="0.511806"/>
   <pageSetup paperSize="1" orientation="portrait" useFirstPageNumber="1"/>

</xml_diff>